<commit_message>
Add assumptions log and interview notes
</commit_message>
<xml_diff>
--- a/docs/assumptions-log.xlsx
+++ b/docs/assumptions-log.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\butcher-price-calculator\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BAD60E2-F97E-4D9C-9878-6E8EA826D74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42129168-5BF3-40D1-AA35-7D33E43A484B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
     <sheet name="Assumptions" sheetId="2" r:id="rId2"/>
     <sheet name="Interview notes" sheetId="3" r:id="rId3"/>
+    <sheet name="Features" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="167">
   <si>
     <t>Assumptions log and interview notes - Butcher price app</t>
   </si>
@@ -184,9 +185,6 @@
     <t>Urdu labels become a must-have</t>
   </si>
   <si>
-    <t>He quotes per kg in whole rupees, rounding halves up</t>
-  </si>
-  <si>
     <t>Rounding rule is wrong, prices are off</t>
   </si>
   <si>
@@ -202,9 +200,6 @@
     <t>Ask Q9</t>
   </si>
   <si>
-    <t>A live bird rate is normally between 200 and 800 PKR/kg</t>
-  </si>
-  <si>
     <t>Typo warning thresholds are wrong</t>
   </si>
   <si>
@@ -361,14 +356,200 @@
     <t>Yes, we trust it and this is the usual way.</t>
   </si>
   <si>
-    <t>I use</t>
+    <t>I use calculator to figure out prices for different cuts based on the live chicken rate.</t>
+  </si>
+  <si>
+    <t>He can make mistake during calculation.</t>
+  </si>
+  <si>
+    <t>Last Friday and cost me 4500 by the end of the day.</t>
+  </si>
+  <si>
+    <t>Their should be a confirmation message when he inputs rate.</t>
+  </si>
+  <si>
+    <t>15 days ago and my previous calculation was wrong.</t>
+  </si>
+  <si>
+    <t>It's only me.</t>
+  </si>
+  <si>
+    <t>Just for information and looking at the trend</t>
+  </si>
+  <si>
+    <t>Yes, I was missed a zero. It remains between 200 to 700 as per my knowledge of last 3 years.</t>
+  </si>
+  <si>
+    <t>My mobile phone and english only.</t>
+  </si>
+  <si>
+    <t>I tell them when they arrive at counter and also send them over the message in WhatsApp.</t>
+  </si>
+  <si>
+    <t>An option to copy the current prices from the app. So he can just past in the message would be a great easy.</t>
+  </si>
+  <si>
+    <t>Nothing bad, it's ok</t>
+  </si>
+  <si>
+    <t>I got it from supplier through a message.</t>
+  </si>
+  <si>
+    <t>He quotes per kg in whole rupees, rounding to nearset 10 ruppee. Five or above means round up.</t>
+  </si>
+  <si>
+    <t>A live bird rate is normally between 200 and 700 PKR/kg</t>
+  </si>
+  <si>
+    <t>Opens early</t>
+  </si>
+  <si>
+    <t>factors entered were not accurate and earn low margin.</t>
+  </si>
+  <si>
+    <t>Make it only for owner.</t>
+  </si>
+  <si>
+    <t>seems not very important</t>
+  </si>
+  <si>
+    <t>Implementing a range check will avoid chances of error.</t>
+  </si>
+  <si>
+    <t>He has to bring movile phone in front of customers frequently.</t>
+  </si>
+  <si>
+    <t>nothing</t>
+  </si>
+  <si>
+    <t>customer trusts on the price quoted by owner.</t>
+  </si>
+  <si>
+    <t>I am buying from this owner for years. I trust</t>
+  </si>
+  <si>
+    <t>Pain (from his words)</t>
+  </si>
+  <si>
+    <t>Feature idea</t>
+  </si>
+  <si>
+    <t>Priority (Must / Should / Could / Won’t now)</t>
+  </si>
+  <si>
+    <t>Why</t>
+  </si>
+  <si>
+    <t>Features</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>F2</t>
+  </si>
+  <si>
+    <t>F3</t>
+  </si>
+  <si>
+    <t>F4</t>
+  </si>
+  <si>
+    <t>F5</t>
+  </si>
+  <si>
+    <t>F6</t>
+  </si>
+  <si>
+    <t>F7</t>
+  </si>
+  <si>
+    <t>F8</t>
+  </si>
+  <si>
+    <t>F9</t>
+  </si>
+  <si>
+    <t>F10</t>
+  </si>
+  <si>
+    <t>F11</t>
+  </si>
+  <si>
+    <t>F12</t>
+  </si>
+  <si>
+    <t>Message to verify if prices are updaed for today in the morning.</t>
+  </si>
+  <si>
+    <t>A check if the entered prices are correct.</t>
+  </si>
+  <si>
+    <t>A check if factors are correct</t>
+  </si>
+  <si>
+    <t>Prices are entered by owner only, no other.</t>
+  </si>
+  <si>
+    <t>nice to have historic trend</t>
+  </si>
+  <si>
+    <t>A confirmation or review about the price entered of the live bird rate.</t>
+  </si>
+  <si>
+    <t>See if prices can be presented independent of the owner's phone. So multiple customers can see the prices instead of looking at the owner's phone.</t>
+  </si>
+  <si>
+    <t>Copy today's price like a message to be copied into the WhatsApp chat is a good option to save owner's time.</t>
+  </si>
+  <si>
+    <t>Must</t>
+  </si>
+  <si>
+    <t>Because if he forget to update, he will loose margins.</t>
+  </si>
+  <si>
+    <t>A wrong prices will be a big loss.</t>
+  </si>
+  <si>
+    <t>Incorrect factors will calculate wrong prices.</t>
+  </si>
+  <si>
+    <t>If prices are entered by anyone else he can fraude the business.</t>
+  </si>
+  <si>
+    <t>Won't now</t>
+  </si>
+  <si>
+    <t>not important</t>
+  </si>
+  <si>
+    <t>Again will be a margin loss.</t>
+  </si>
+  <si>
+    <t>Should</t>
+  </si>
+  <si>
+    <t>Owner can use his phone and customers should be able to know prices from location recommended by owner.</t>
+  </si>
+  <si>
+    <t>I can't entere prices directly. It always comes from factors.</t>
+  </si>
+  <si>
+    <t>Cut prices should be entered directly overiding factors through a button option.</t>
+  </si>
+  <si>
+    <t>sometimes it’s difficult to get optimized prices through factors.</t>
+  </si>
+  <si>
+    <t>To save owners time over the call or writing message in the WhatsApp</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -417,6 +598,12 @@
       <sz val="10"/>
       <color rgb="FF7F7F7F"/>
       <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -935,7 +1122,7 @@
       </c>
       <c r="C3" s="8">
         <f>COUNTIF(D8:D37,"Verified")</f>
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -944,7 +1131,7 @@
       </c>
       <c r="C4" s="8">
         <f>COUNTIF(D8:D37,"Guess")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -1060,9 +1247,11 @@
       <c r="B11" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="11"/>
+      <c r="C11" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="D11" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>37</v>
@@ -1083,9 +1272,11 @@
       <c r="B12" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="11"/>
+      <c r="C12" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="D12" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>40</v>
@@ -1106,9 +1297,11 @@
       <c r="B13" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="11"/>
+      <c r="C13" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="D13" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>43</v>
@@ -1129,9 +1322,11 @@
       <c r="B14" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="11"/>
+      <c r="C14" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="D14" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>46</v>
@@ -1144,23 +1339,25 @@
         <v>OK</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="25" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="str">
         <f t="shared" si="0"/>
         <v>A8</v>
       </c>
       <c r="B15" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="E15" s="10" t="s">
+      <c r="F15" s="10" t="s">
         <v>48</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>49</v>
       </c>
       <c r="G15" s="10" t="str">
         <f t="shared" si="1"/>
@@ -1173,17 +1370,19 @@
         <v>A9</v>
       </c>
       <c r="B16" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="10" t="s">
         <v>51</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>52</v>
       </c>
       <c r="G16" s="10" t="str">
         <f t="shared" si="1"/>
@@ -1196,17 +1395,19 @@
         <v>A10</v>
       </c>
       <c r="B17" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F17" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>55</v>
       </c>
       <c r="G17" s="10" t="str">
         <f t="shared" si="1"/>
@@ -1219,17 +1420,17 @@
         <v>A11</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C18" s="11"/>
       <c r="D18" s="11" t="s">
         <v>16</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G18" s="10" t="str">
         <f t="shared" si="1"/>
@@ -1564,12 +1765,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="20" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B2" s="14">
         <v>46310</v>
@@ -1577,198 +1778,470 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="26" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="D6" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="E6" s="9" t="s">
         <v>65</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="62.5" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>68</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="D7" s="11"/>
-      <c r="E7" s="10" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>71</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="D8" s="11"/>
-      <c r="E8" s="10" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>74</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="10" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="10" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="E11" s="10" t="s">
         <v>80</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="10" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="E12" s="10" t="s">
         <v>83</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="10" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="E13" s="10" t="s">
         <v>86</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="10" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="E14" s="10" t="s">
         <v>89</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="10" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>92</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="10" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>95</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="10" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="E17" s="10" t="s">
         <v>98</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="10" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D18" s="11"/>
+        <v>103</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>127</v>
+      </c>
       <c r="E18" s="10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53BBB129-0318-4E8E-BFEE-73C963F89362}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="6.6328125" customWidth="1"/>
+    <col min="2" max="3" width="48" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="20" x14ac:dyDescent="0.4">
+      <c r="A1" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="39" x14ac:dyDescent="0.35">
+      <c r="A3" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="25" x14ac:dyDescent="0.35">
+      <c r="A4" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="25" x14ac:dyDescent="0.35">
+      <c r="A6" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="25" x14ac:dyDescent="0.35">
+      <c r="A7" s="10"/>
+      <c r="B7" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="25" x14ac:dyDescent="0.35">
+      <c r="A8" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="25" x14ac:dyDescent="0.35">
+      <c r="A10" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="25" x14ac:dyDescent="0.35">
+      <c r="A12" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
 </file>
</xml_diff>